<commit_message>
doin some more interview prep
</commit_message>
<xml_diff>
--- a/job_tracker/job_search_tracker.xlsx
+++ b/job_tracker/job_search_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n0308g\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F10425FF-1700-4AA5-8A47-EB5D8424DDD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D34096-A87D-4E85-BC25-4CF7554320D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="118">
   <si>
     <t>Job Search Tracker — How to Use</t>
   </si>
@@ -328,15 +328,9 @@
     <t>https://job-boards.greenhouse.io/rackner/jobs/4702089005</t>
   </si>
   <si>
-    <t>Erica Hakim</t>
-  </si>
-  <si>
     <t>Talent Acquisition Advisor</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/erica-hakim-3aa33161/</t>
-  </si>
-  <si>
     <t>Healthcare Privacy &amp; Compliance Leader</t>
   </si>
   <si>
@@ -383,6 +377,21 @@
   </si>
   <si>
     <t>https://careers.mantech.com/en_US/careers/JobDetail/63865?source=appcast_Linkedin_Sponsored&amp;_ccid=1783639067959w7ieki6f7&amp;__ssr=true</t>
+  </si>
+  <si>
+    <t>Erica Hakim, Amerlia Davenport</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/erica-hakim-3aa33161/, https://www.linkedin.com/in/amelia-davenport/</t>
+  </si>
+  <si>
+    <t>Erica Hakim, Amelia Davenport</t>
+  </si>
+  <si>
+    <t>AI Software Engineer</t>
+  </si>
+  <si>
+    <t>https://guidehouse.wd1.myworkdayjobs.com/en-US/External/job/AI-Software-Engineer_40569</t>
   </si>
 </sst>
 </file>
@@ -392,13 +401,20 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -529,62 +545,65 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -986,7 +1005,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O300"/>
+  <dimension ref="A1:O301"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1118,14 +1137,14 @@
       <c r="F3" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="G3" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="H3" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="H3" s="15" t="s">
-        <v>97</v>
-      </c>
       <c r="I3" s="15" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="J3" s="17">
         <v>46213</v>
@@ -1161,14 +1180,14 @@
       <c r="F4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="G4" s="21" t="s">
+      <c r="G4" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="H4" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="H4" s="15" t="s">
-        <v>97</v>
-      </c>
       <c r="I4" s="15" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="J4" s="17">
         <v>46213</v>
@@ -1192,32 +1211,32 @@
       <c r="B5" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="21" t="s">
-        <v>77</v>
+      <c r="C5" s="23" t="s">
+        <v>116</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>75</v>
+        <v>117</v>
       </c>
       <c r="E5" s="17">
-        <v>46211</v>
+        <v>46216</v>
       </c>
       <c r="F5" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="G5" s="15" t="s">
-        <v>73</v>
+      <c r="G5" s="23" t="s">
+        <v>115</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>73</v>
+        <v>114</v>
+      </c>
+      <c r="J5" s="17">
+        <v>46213</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="L5" s="15" t="s">
         <v>73</v>
@@ -1228,24 +1247,24 @@
       <c r="N5" s="15"/>
       <c r="O5" s="15"/>
     </row>
-    <row r="6" spans="1:15" ht="195" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" ht="232" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>79</v>
+        <v>69</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>75</v>
       </c>
       <c r="E6" s="17">
-        <v>46203</v>
+        <v>46211</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="G6" s="15" t="s">
         <v>73</v>
@@ -1271,24 +1290,24 @@
       <c r="N6" s="15"/>
       <c r="O6" s="15"/>
     </row>
-    <row r="7" spans="1:15" ht="286" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" ht="195" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>79</v>
       </c>
       <c r="E7" s="17">
         <v>46203</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>73</v>
@@ -1314,39 +1333,39 @@
       <c r="N7" s="15"/>
       <c r="O7" s="15"/>
     </row>
-    <row r="8" spans="1:15" ht="377" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" ht="286" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E8" s="17">
-        <v>46212</v>
+        <v>46203</v>
       </c>
       <c r="F8" s="15" t="s">
         <v>40</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>109</v>
+        <v>73</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="J8" s="17">
-        <v>46213</v>
+        <v>73</v>
+      </c>
+      <c r="J8" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="L8" s="15" t="s">
         <v>73</v>
@@ -1355,9 +1374,7 @@
         <v>73</v>
       </c>
       <c r="N8" s="15"/>
-      <c r="O8" s="15" t="s">
-        <v>107</v>
-      </c>
+      <c r="O8" s="15"/>
     </row>
     <row r="9" spans="1:15" ht="377" x14ac:dyDescent="0.35">
       <c r="A9" s="15" t="s">
@@ -1367,10 +1384,10 @@
         <v>90</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E9" s="17">
         <v>46212</v>
@@ -1379,13 +1396,13 @@
         <v>40</v>
       </c>
       <c r="G9" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="I9" s="15" t="s">
         <v>108</v>
-      </c>
-      <c r="H9" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="I9" s="15" t="s">
-        <v>110</v>
       </c>
       <c r="J9" s="17">
         <v>46213</v>
@@ -1401,21 +1418,21 @@
       </c>
       <c r="N9" s="15"/>
       <c r="O9" s="15" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" ht="234" x14ac:dyDescent="0.35">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="377" x14ac:dyDescent="0.35">
       <c r="A10" s="15" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E10" s="17">
         <v>46212</v>
@@ -1424,19 +1441,19 @@
         <v>40</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="J10" s="15" t="s">
-        <v>73</v>
+        <v>108</v>
+      </c>
+      <c r="J10" s="17">
+        <v>46213</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="L10" s="15" t="s">
         <v>73</v>
@@ -1445,25 +1462,27 @@
         <v>73</v>
       </c>
       <c r="N10" s="15"/>
-      <c r="O10" s="15"/>
-    </row>
-    <row r="11" spans="1:15" ht="187.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="B11" s="14" t="s">
+      <c r="O10" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="E11" s="13">
-        <v>46213</v>
-      </c>
-      <c r="F11" s="3" t="s">
+    </row>
+    <row r="11" spans="1:15" ht="234" x14ac:dyDescent="0.35">
+      <c r="A11" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" s="17">
+        <v>46212</v>
+      </c>
+      <c r="F11" s="15" t="s">
         <v>40</v>
       </c>
       <c r="G11" s="15" t="s">
@@ -1487,27 +1506,27 @@
       <c r="M11" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-    </row>
-    <row r="12" spans="1:15" ht="325" x14ac:dyDescent="0.35">
+      <c r="N11" s="15"/>
+      <c r="O11" s="15"/>
+    </row>
+    <row r="12" spans="1:15" ht="187.5" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>106</v>
+        <v>100</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>103</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>73</v>
+        <v>99</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="E12" s="13">
-        <v>46195</v>
+        <v>46213</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>73</v>
@@ -1533,24 +1552,24 @@
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
     </row>
-    <row r="13" spans="1:15" ht="350" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" ht="325" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>114</v>
+        <v>101</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>73</v>
       </c>
       <c r="E13" s="13">
-        <v>46213</v>
+        <v>46195</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="G13" s="15" t="s">
         <v>73</v>
@@ -1576,20 +1595,46 @@
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
+    <row r="14" spans="1:15" ht="350" x14ac:dyDescent="0.35">
+      <c r="A14" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="13">
+        <v>46213</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="K14" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="L14" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="M14" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
     </row>
@@ -6455,27 +6500,44 @@
       <c r="N300" s="3"/>
       <c r="O300" s="3"/>
     </row>
+    <row r="301" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A301" s="3"/>
+      <c r="B301" s="3"/>
+      <c r="C301" s="3"/>
+      <c r="D301" s="3"/>
+      <c r="E301" s="3"/>
+      <c r="F301" s="3"/>
+      <c r="G301" s="3"/>
+      <c r="H301" s="3"/>
+      <c r="I301" s="3"/>
+      <c r="J301" s="3"/>
+      <c r="K301" s="3"/>
+      <c r="L301" s="3"/>
+      <c r="M301" s="3"/>
+      <c r="N301" s="3"/>
+      <c r="O301" s="3"/>
+    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" sqref="F3:F300" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F3:F301" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Not Applied,Applied,Phone Screen,Technical Interview,Onsite/Final,Offer,Rejected,Withdrawn"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="K3:K5 K14:K300" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="K15:K301 K3:K6" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Not Contacted,Messaged,Replied,Call Scheduled,Call Completed,Referred,No Response"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L3:L5 L14:L300" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="L15:L301 L3:L6" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Yes,No,Pending"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="N3:N300" xr:uid="{00000000-0002-0000-0100-000003000000}">
+    <dataValidation type="list" allowBlank="1" sqref="N3:N301" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D6" r:id="rId1" xr:uid="{101B10EA-B6F9-48E5-BF9A-79BA2B6FB2AD}"/>
+    <hyperlink ref="D7" r:id="rId1" xr:uid="{101B10EA-B6F9-48E5-BF9A-79BA2B6FB2AD}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6519,14 +6581,14 @@
         <v>52</v>
       </c>
       <c r="B5" s="8">
-        <f>COUNTIF('Job Tracker'!F3:F300,"Not Applied")</f>
+        <f>COUNTIF('Job Tracker'!F3:F301,"Not Applied")</f>
         <v>0</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>53</v>
       </c>
       <c r="E5" s="8">
-        <f>COUNTIF('Job Tracker'!K3:K300,"Not Contacted")</f>
+        <f>COUNTIF('Job Tracker'!K3:K301,"Not Contacted")</f>
         <v>0</v>
       </c>
     </row>
@@ -6535,15 +6597,15 @@
         <v>40</v>
       </c>
       <c r="B6" s="8">
-        <f>COUNTIF('Job Tracker'!F3:F300,"Applied")</f>
-        <v>9</v>
+        <f>COUNTIF('Job Tracker'!F3:F301,"Applied")</f>
+        <v>10</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>45</v>
       </c>
       <c r="E6" s="8">
-        <f>COUNTIF('Job Tracker'!K3:K300,"Messaged")</f>
-        <v>2</v>
+        <f>COUNTIF('Job Tracker'!K3:K301,"Messaged")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -6551,14 +6613,14 @@
         <v>54</v>
       </c>
       <c r="B7" s="8">
-        <f>COUNTIF('Job Tracker'!F3:F300,"Phone Screen")</f>
+        <f>COUNTIF('Job Tracker'!F3:F301,"Phone Screen")</f>
         <v>0</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>55</v>
       </c>
       <c r="E7" s="8">
-        <f>COUNTIF('Job Tracker'!K3:K300,"Replied")</f>
+        <f>COUNTIF('Job Tracker'!K3:K301,"Replied")</f>
         <v>2</v>
       </c>
     </row>
@@ -6567,14 +6629,14 @@
         <v>56</v>
       </c>
       <c r="B8" s="8">
-        <f>COUNTIF('Job Tracker'!F3:F300,"Technical Interview")</f>
+        <f>COUNTIF('Job Tracker'!F3:F301,"Technical Interview")</f>
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>57</v>
       </c>
       <c r="E8" s="8">
-        <f>COUNTIF('Job Tracker'!K3:K300,"Call Scheduled")</f>
+        <f>COUNTIF('Job Tracker'!K3:K301,"Call Scheduled")</f>
         <v>0</v>
       </c>
     </row>
@@ -6583,14 +6645,14 @@
         <v>58</v>
       </c>
       <c r="B9" s="8">
-        <f>COUNTIF('Job Tracker'!F3:F300,"Onsite/Final")</f>
+        <f>COUNTIF('Job Tracker'!F3:F301,"Onsite/Final")</f>
         <v>0</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>59</v>
       </c>
       <c r="E9" s="8">
-        <f>COUNTIF('Job Tracker'!K3:K300,"Call Completed")</f>
+        <f>COUNTIF('Job Tracker'!K3:K301,"Call Completed")</f>
         <v>0</v>
       </c>
     </row>
@@ -6599,14 +6661,14 @@
         <v>60</v>
       </c>
       <c r="B10" s="8">
-        <f>COUNTIF('Job Tracker'!F3:F300,"Offer")</f>
+        <f>COUNTIF('Job Tracker'!F3:F301,"Offer")</f>
         <v>0</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>61</v>
       </c>
       <c r="E10" s="8">
-        <f>COUNTIF('Job Tracker'!K3:K300,"Referred")</f>
+        <f>COUNTIF('Job Tracker'!K3:K301,"Referred")</f>
         <v>0</v>
       </c>
     </row>
@@ -6615,14 +6677,14 @@
         <v>62</v>
       </c>
       <c r="B11" s="8">
-        <f>COUNTIF('Job Tracker'!F3:F300,"Rejected")</f>
+        <f>COUNTIF('Job Tracker'!F3:F301,"Rejected")</f>
         <v>2</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>63</v>
       </c>
       <c r="E11" s="8">
-        <f>COUNTIF('Job Tracker'!K3:K300,"No Response")</f>
+        <f>COUNTIF('Job Tracker'!K3:K301,"No Response")</f>
         <v>0</v>
       </c>
     </row>
@@ -6631,7 +6693,7 @@
         <v>64</v>
       </c>
       <c r="B12" s="8">
-        <f>COUNTIF('Job Tracker'!F3:F300,"Withdrawn")</f>
+        <f>COUNTIF('Job Tracker'!F3:F301,"Withdrawn")</f>
         <v>0</v>
       </c>
     </row>
@@ -6640,15 +6702,15 @@
         <v>65</v>
       </c>
       <c r="B13" s="10">
-        <f>COUNTA('Job Tracker'!A3:A300)</f>
-        <v>11</v>
+        <f>COUNTA('Job Tracker'!A3:A301)</f>
+        <v>12</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>66</v>
       </c>
       <c r="E13" s="11">
-        <f>IFERROR(COUNTIF('Job Tracker'!K3:K300,"Replied")/(COUNTA('Job Tracker'!K3:K300)-COUNTIF('Job Tracker'!K3:K300,"Not Contacted")),0)</f>
-        <v>0.18181818181818182</v>
+        <f>IFERROR(COUNTIF('Job Tracker'!K3:K301,"Replied")/(COUNTA('Job Tracker'!K3:K301)-COUNTIF('Job Tracker'!K3:K301,"Not Contacted")),0)</f>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -6656,7 +6718,7 @@
         <v>67</v>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIF('Job Tracker'!L3:L300,"Yes")</f>
+        <f>COUNTIF('Job Tracker'!L3:L301,"Yes")</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
zip zip zip dooba doobadooba
</commit_message>
<xml_diff>
--- a/job_tracker/job_search_tracker.xlsx
+++ b/job_tracker/job_search_tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n0308g\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n0308g\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D34096-A87D-4E85-BC25-4CF7554320D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18568651-A530-40DE-9137-B90BBBBE4104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3840" yWindow="240" windowWidth="21600" windowHeight="20970" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="137">
   <si>
     <t>Job Search Tracker — How to Use</t>
   </si>
@@ -392,6 +392,63 @@
   </si>
   <si>
     <t>https://guidehouse.wd1.myworkdayjobs.com/en-US/External/job/AI-Software-Engineer_40569</t>
+  </si>
+  <si>
+    <t>Lockheed Martin</t>
+  </si>
+  <si>
+    <t>You know</t>
+  </si>
+  <si>
+    <t>AI/Machine Learning Engineer Senior</t>
+  </si>
+  <si>
+    <t>https://www.lockheedmartinjobs.com/job/grand-prairie/ai-machine-learning-engineer-senior/694/95959930352</t>
+  </si>
+  <si>
+    <t>https://www.lockheedmartinjobs.com/job/grand-prairie/supply-chain-ai-developer/694/96206196960</t>
+  </si>
+  <si>
+    <t>Supply Chain AI Developer</t>
+  </si>
+  <si>
+    <t>Booz Allen Hamilton is a management and technology consulting firm that primarily serves the U.S. government, especially defense, intelligence, and federal agencies. It focuses on areas like cybersecurity, IT/digital transformation, data analytics, and engineering, alongside some commercial and international clients.</t>
+  </si>
+  <si>
+    <t>Booz Allen Hamilton</t>
+  </si>
+  <si>
+    <t>AI Developer</t>
+  </si>
+  <si>
+    <t>AI Engineer</t>
+  </si>
+  <si>
+    <t>https://bah.wd1.myworkdayjobs.com/en-US/BAH_Jobs/job/AI-Engineer_R0241255</t>
+  </si>
+  <si>
+    <t>https://bah.wd1.myworkdayjobs.com/en-US/BAH_Jobs/job/AI-Developer_R0243553</t>
+  </si>
+  <si>
+    <t>Talked with a data science consultant, Amelia &lt;something&gt;. They seem pretty chill.</t>
+  </si>
+  <si>
+    <t>https://jobs.northropgrumman.com/careers/job/1340072851428?code=JB-18202&amp;domain=ngc.com&amp;rx_campaign=Linkedin1&amp;rx_ch=connector&amp;rx_group=375073&amp;rx_id=a4421b8b-7d26-11f1-94f1-2d7da755d61b&amp;rx_job=R10239479&amp;rx_medium=post&amp;rx_r=none&amp;rx_source=Linkedin&amp;rx_vp=slots&amp;source=JB-18202&amp;utm_audience=prospectivetalentemployees&amp;utm_campaign=ta-general&amp;utm_content=jobfeed&amp;utm_format=cpl&amp;utm_medium=jobboard&amp;utm_network=partnerdirect&amp;utm_source=linkedin-jobslots&amp;rx_viewer=5f582f71f8b111f0a982077e321431c66e3f1f5429d9445b97cce3715703767b</t>
+  </si>
+  <si>
+    <t>Principal/Sr Principal Software Engineer</t>
+  </si>
+  <si>
+    <t>Northrup Grumman</t>
+  </si>
+  <si>
+    <t>This role become no longer available so I was rejected because of that.</t>
+  </si>
+  <si>
+    <t>Recruiter called 8/31/2026. Potential interview pending, with them knowin the 135k target. However, I may be able to leverage off of NG to get this number higher.</t>
+  </si>
+  <si>
+    <t>Verbal offer given July 30th. 129k and 10k sign-on bonus. Negotiated for 135k, and it's been about 1 month since then.  Didn't work out to 135k. Offer accepted at 129k with the 10k sign on bonus. Tenative start state September 21st, 2026.</t>
   </si>
 </sst>
 </file>
@@ -547,7 +604,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -597,13 +654,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1137,7 +1191,7 @@
       <c r="F3" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="G3" s="23" t="s">
+      <c r="G3" s="22" t="s">
         <v>113</v>
       </c>
       <c r="H3" s="15" t="s">
@@ -1180,7 +1234,7 @@
       <c r="F4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="G4" s="23" t="s">
+      <c r="G4" s="22" t="s">
         <v>115</v>
       </c>
       <c r="H4" s="15" t="s">
@@ -1211,7 +1265,7 @@
       <c r="B5" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="22" t="s">
         <v>116</v>
       </c>
       <c r="D5" s="15" t="s">
@@ -1223,7 +1277,7 @@
       <c r="F5" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="G5" s="22" t="s">
         <v>115</v>
       </c>
       <c r="H5" s="15" t="s">
@@ -1245,7 +1299,9 @@
         <v>73</v>
       </c>
       <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
+      <c r="O5" s="15" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="6" spans="1:15" ht="232" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
@@ -1288,7 +1344,9 @@
         <v>73</v>
       </c>
       <c r="N6" s="15"/>
-      <c r="O6" s="15"/>
+      <c r="O6" s="15" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="7" spans="1:15" ht="195" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
@@ -1297,7 +1355,7 @@
       <c r="B7" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="21" t="s">
         <v>80</v>
       </c>
       <c r="D7" s="18" t="s">
@@ -1638,90 +1696,225 @@
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
+    <row r="15" spans="1:15" ht="62.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E15" s="13">
+        <v>46224</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="J15" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="K15" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="M15" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
+    <row r="16" spans="1:15" ht="62.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E16" s="13">
+        <v>46224</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="L16" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="M16" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
+    <row r="17" spans="1:15" ht="150" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E17" s="13">
+        <v>46224</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="L17" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="N17" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="150" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E18" s="13">
+        <v>46224</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="J18" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="K18" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="L18" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="M18" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
+      <c r="O18" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="312.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E19" s="13">
+        <v>46226</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="J19" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="K19" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="L19" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="M19" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
+      <c r="O19" s="3" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
@@ -6523,11 +6716,11 @@
       <formula1>"Not Applied,Applied,Phone Screen,Technical Interview,Onsite/Final,Offer,Rejected,Withdrawn"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="K15:K301 K3:K6" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="K3:K6 K20:K301" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Not Contacted,Messaged,Replied,Call Scheduled,Call Completed,Referred,No Response"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L15:L301 L3:L6" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="L3:L6 L20:L301" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Yes,No,Pending"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6540,7 +6733,7 @@
     <hyperlink ref="D7" r:id="rId1" xr:uid="{101B10EA-B6F9-48E5-BF9A-79BA2B6FB2AD}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -6598,7 +6791,7 @@
       </c>
       <c r="B6" s="8">
         <f>COUNTIF('Job Tracker'!F3:F301,"Applied")</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>45</v>
@@ -6662,7 +6855,7 @@
       </c>
       <c r="B10" s="8">
         <f>COUNTIF('Job Tracker'!F3:F301,"Offer")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>61</v>
@@ -6678,7 +6871,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF('Job Tracker'!F3:F301,"Rejected")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>63</v>
@@ -6703,14 +6896,14 @@
       </c>
       <c r="B13" s="10">
         <f>COUNTA('Job Tracker'!A3:A301)</f>
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>66</v>
       </c>
       <c r="E13" s="11">
         <f>IFERROR(COUNTIF('Job Tracker'!K3:K301,"Replied")/(COUNTA('Job Tracker'!K3:K301)-COUNTIF('Job Tracker'!K3:K301,"Not Contacted")),0)</f>
-        <v>0.16666666666666666</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>